<commit_message>
feat(core): implementar servicio institucional de folios
</commit_message>
<xml_diff>
--- a/importaciones/tesoreria/TESORERIA_MOVIMIENTOS_2026.xlsx
+++ b/importaciones/tesoreria/TESORERIA_MOVIMIENTOS_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="15"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="14"/>
   </bookViews>
   <sheets>
     <sheet name="MIEMBROS" sheetId="1" state="visible" r:id="rId3"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="433">
   <si>
     <t xml:space="preserve">ID_MIEMBRO</t>
   </si>
@@ -912,6 +912,21 @@
   </si>
   <si>
     <t xml:space="preserve">USR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consecutivo de recibos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consecutivo de pagos</t>
   </si>
   <si>
     <t xml:space="preserve">CATALOGO</t>
@@ -1335,7 +1350,7 @@
     <numFmt numFmtId="169" formatCode="m/d/yyyy\ h:mm:ss"/>
     <numFmt numFmtId="170" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1396,6 +1411,13 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1439,7 +1461,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1534,6 +1556,10 @@
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -3087,16 +3113,34 @@
       <c r="E30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
+      <c r="A31" s="24" t="s">
+        <v>292</v>
+      </c>
+      <c r="B31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="0"/>
+      <c r="D31" s="24" t="s">
+        <v>293</v>
+      </c>
+      <c r="E31" s="24" t="s">
+        <v>294</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
+      <c r="A32" s="24" t="s">
+        <v>295</v>
+      </c>
+      <c r="B32" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="0"/>
+      <c r="D32" s="24" t="s">
+        <v>296</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>294</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="6"/>
@@ -8903,10 +8947,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>239</v>
@@ -8920,13 +8964,13 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>134</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="5" t="s">
@@ -8935,13 +8979,13 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="5" t="s">
@@ -8950,13 +8994,13 @@
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="5" t="s">
@@ -8965,13 +9009,13 @@
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>133</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="5" t="s">
@@ -8980,13 +9024,13 @@
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="5" t="s">
@@ -8995,13 +9039,13 @@
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="5" t="s">
@@ -9010,13 +9054,13 @@
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>140</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="5" t="s">
@@ -9025,13 +9069,13 @@
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="5" t="s">
@@ -9040,13 +9084,13 @@
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="5" t="s">
@@ -9055,13 +9099,13 @@
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="5" t="s">
@@ -9070,13 +9114,13 @@
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="5" t="s">
@@ -9085,13 +9129,13 @@
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="5" t="s">
@@ -9100,13 +9144,13 @@
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="5" t="s">
@@ -9115,13 +9159,13 @@
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="5" t="s">
@@ -9130,13 +9174,13 @@
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="5" t="s">
@@ -9145,13 +9189,13 @@
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="5" t="s">
@@ -9160,13 +9204,13 @@
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="5" t="s">
@@ -9175,13 +9219,13 @@
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="5" t="s">
@@ -9190,13 +9234,13 @@
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="5" t="s">
@@ -9205,13 +9249,13 @@
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="5" t="s">
@@ -9223,10 +9267,10 @@
         <v>159</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="5" t="s">
@@ -9238,10 +9282,10 @@
         <v>159</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="5" t="s">
@@ -9253,10 +9297,10 @@
         <v>159</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="5" t="s">
@@ -9268,10 +9312,10 @@
         <v>159</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="5" t="s">
@@ -9280,13 +9324,13 @@
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>203</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="5" t="s">
@@ -9295,13 +9339,13 @@
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="5" t="s">
@@ -9310,13 +9354,13 @@
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="D28" s="6"/>
       <c r="E28" s="5" t="s">
@@ -9325,13 +9369,13 @@
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>180</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="5" t="s">
@@ -9340,7 +9384,7 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>182</v>
@@ -9351,7 +9395,7 @@
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>184</v>
@@ -9362,7 +9406,7 @@
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>186</v>
@@ -9373,7 +9417,7 @@
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>188</v>
@@ -9384,10 +9428,10 @@
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="6"/>
@@ -9395,7 +9439,7 @@
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>190</v>
@@ -9406,7 +9450,7 @@
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>192</v>
@@ -9417,7 +9461,7 @@
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>194</v>
@@ -9428,7 +9472,7 @@
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>196</v>
@@ -9439,7 +9483,7 @@
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>198</v>
@@ -9450,7 +9494,7 @@
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>200</v>
@@ -9461,7 +9505,7 @@
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>202</v>
@@ -9472,10 +9516,10 @@
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="6"/>
@@ -9483,10 +9527,10 @@
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="6"/>
@@ -9494,10 +9538,10 @@
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="6"/>
@@ -9505,10 +9549,10 @@
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="6"/>
@@ -9516,10 +9560,10 @@
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="6"/>
@@ -9527,10 +9571,10 @@
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="C47" s="5"/>
       <c r="D47" s="6"/>
@@ -9538,10 +9582,10 @@
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="6"/>
@@ -9549,10 +9593,10 @@
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="6"/>
@@ -9560,10 +9604,10 @@
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="6"/>
@@ -9571,10 +9615,10 @@
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>59</v>
@@ -9588,10 +9632,10 @@
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>46</v>
@@ -9605,10 +9649,10 @@
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="C53" s="5" t="s">
         <v>27</v>
@@ -9625,10 +9669,10 @@
         <v>19</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="D54" s="6"/>
     </row>
@@ -9637,10 +9681,10 @@
         <v>19</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="D55" s="6"/>
     </row>
@@ -9649,10 +9693,10 @@
         <v>19</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="D56" s="6"/>
     </row>
@@ -9661,10 +9705,10 @@
         <v>19</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="D57" s="6"/>
     </row>
@@ -9673,70 +9717,70 @@
         <v>19</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="D58" s="6"/>
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>134</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="D59" s="6"/>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="D60" s="6"/>
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="D61" s="6"/>
     </row>
     <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="D62" s="6"/>
     </row>
     <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D63" s="6" t="n">
         <v>1</v>
@@ -9747,13 +9791,13 @@
     </row>
     <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="D64" s="6" t="n">
         <v>2</v>
@@ -9764,13 +9808,13 @@
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="D65" s="6" t="n">
         <v>3</v>
@@ -9781,13 +9825,13 @@
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="D66" s="6" t="n">
         <v>4</v>
@@ -9798,13 +9842,13 @@
     </row>
     <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="D67" s="6" t="n">
         <v>5</v>
@@ -9815,13 +9859,13 @@
     </row>
     <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="D68" s="6" t="n">
         <v>6</v>
@@ -9832,13 +9876,13 @@
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="D69" s="6" t="n">
         <v>7</v>
@@ -9849,13 +9893,13 @@
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="D70" s="6" t="n">
         <v>8</v>
@@ -9866,13 +9910,13 @@
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="D71" s="6" t="n">
         <v>9</v>
@@ -9883,13 +9927,13 @@
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="D72" s="6" t="n">
         <v>10</v>
@@ -9900,13 +9944,13 @@
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="D73" s="6" t="n">
         <v>11</v>
@@ -9917,13 +9961,13 @@
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="D74" s="6" t="n">
         <v>12</v>
@@ -9934,13 +9978,13 @@
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>180</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="D75" s="6"/>
       <c r="E75" s="5" t="s">
@@ -9949,13 +9993,13 @@
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>182</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="D76" s="6"/>
       <c r="E76" s="5" t="s">
@@ -9964,13 +10008,13 @@
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="D77" s="6"/>
       <c r="E77" s="5" t="s">
@@ -9979,7 +10023,7 @@
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>186</v>
@@ -9994,13 +10038,13 @@
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>188</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="D79" s="6"/>
       <c r="E79" s="5" t="s">
@@ -10009,13 +10053,13 @@
     </row>
     <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>190</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="D80" s="6"/>
       <c r="E80" s="5" t="s">
@@ -10024,13 +10068,13 @@
     </row>
     <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>192</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="D81" s="6"/>
       <c r="E81" s="5" t="s">
@@ -10039,13 +10083,13 @@
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>194</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="D82" s="6"/>
       <c r="E82" s="5" t="s">
@@ -10054,13 +10098,13 @@
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>196</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="D83" s="6"/>
       <c r="E83" s="5" t="s">
@@ -10069,13 +10113,13 @@
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>198</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="D84" s="6"/>
       <c r="E84" s="5" t="s">
@@ -10084,13 +10128,13 @@
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B85" s="5" t="s">
         <v>200</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="D85" s="6"/>
       <c r="E85" s="5" t="s">
@@ -10099,13 +10143,13 @@
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B86" s="5" t="s">
         <v>202</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="D86" s="6"/>
       <c r="E86" s="5" t="s">
@@ -10114,13 +10158,13 @@
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="5" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>203</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="D87" s="6"/>
       <c r="E87" s="5" t="s">
@@ -10129,49 +10173,49 @@
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="5" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="D88" s="6"/>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="5" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="D89" s="6"/>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="5" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="D90" s="6"/>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="5" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="D91" s="6"/>
     </row>
@@ -10205,7 +10249,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>237</v>
@@ -10245,7 +10289,7 @@
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>115</v>
@@ -10253,15 +10297,15 @@
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>46195</v>

</xml_diff>